<commit_message>
Excel-Komfort: Tipp-Birne automatisch, Filter und Emoji-Farbe
- Tipp-Spalte ohne führende 💡 – build.py ergänzt die Birne automatisch
  (idempotent, leerer Tipp bleibt leer)
- AutoFilter (Filter-Pfeile) in der Kopfzeile aller Blätter
- Emoji-/Icon-Spalten in Schriftart "Segoe UI Emoji" für farbige Anzeige
- tools/seed_excel.py: reproduzierbares Neu-Erstellen/Zuruecksetzen der Excel
  aus Skillsliste.html (nur Einrichtung, nicht laufende Pflege)
- ANLEITUNG.md ergaenzt (Tipp-Regel, Filter, Emoji-Farb-Hinweis)

Verifiziert: alle 100 Skills 1:1 wie in der aktuellen Skillsliste.html;
generierte HTML bleibt unveraendert.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills_daten.xlsx
+++ b/skills_daten.xlsx
@@ -11,7 +11,11 @@
     <sheet name="Stufen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Kategorien" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Skills'!$A$1:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stufen'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorien'!$A$1:$C$10</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +34,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Segoe UI Emoji"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -62,7 +70,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -504,7 +512,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>💡 Einfach ein kleines Stück abbeissen und kurz im Mund lassen. 15 – 30 Sekunden genügen.</t>
+          <t>Einfach ein kleines Stück abbeissen und kurz im Mund lassen. 15 – 30 Sekunden genügen.</t>
         </is>
       </c>
     </row>
@@ -536,7 +544,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>💡 Immer ein paar in der Tasche haben — ideal als diskrete Notfalllösung.</t>
+          <t>Immer ein paar in der Tasche haben — ideal als diskrete Notfalllösung.</t>
         </is>
       </c>
     </row>
@@ -568,7 +576,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>💡 Kombination mit Wasabi ergibt noch stärkere Wirkung.</t>
+          <t>Kombination mit Wasabi ergibt noch stärkere Wirkung.</t>
         </is>
       </c>
     </row>
@@ -600,7 +608,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>💡 Kleine Flasche lässt sich leicht mitnehmen.</t>
+          <t>Kleine Flasche lässt sich leicht mitnehmen.</t>
         </is>
       </c>
     </row>
@@ -632,7 +640,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>💡 Nur sehr kleine Menge verwenden. Wirkung tritt innerhalb von Sekunden ein.</t>
+          <t>Nur sehr kleine Menge verwenden. Wirkung tritt innerhalb von Sekunden ein.</t>
         </is>
       </c>
     </row>
@@ -664,7 +672,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>💡 Zitrone in Scheiben schneiden und direkt reinbeissen — oder den Saft auf die Zunge träufeln.</t>
+          <t>Zitrone in Scheiben schneiden und direkt reinbeissen — oder den Saft auf die Zunge träufeln.</t>
         </is>
       </c>
     </row>
@@ -696,7 +704,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>💡 Kurz unter die Nase halten, nicht direkt einatmen.</t>
+          <t>Kurz unter die Nase halten, nicht direkt einatmen.</t>
         </is>
       </c>
     </row>
@@ -728,7 +736,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>💡 Tigerbalm ist handlicher und weniger aggressiv als reines Ammoniak.</t>
+          <t>Tigerbalm ist handlicher und weniger aggressiv als reines Ammoniak.</t>
         </is>
       </c>
     </row>
@@ -760,7 +768,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>💡 Auf Vorrat im Tiefkühler halten. Wirkt besonders gut als Belohnungsritual nach einer überstandenen Krise.</t>
+          <t>Auf Vorrat im Tiefkühler halten. Wirkt besonders gut als Belohnungsritual nach einer überstandenen Krise.</t>
         </is>
       </c>
     </row>
@@ -792,7 +800,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>💡 Nelke wirkt auch leicht betäubend auf die Mundschleimhaut — hilft bei körperlicher Unruhe.</t>
+          <t>Nelke wirkt auch leicht betäubend auf die Mundschleimhaut — hilft bei körperlicher Unruhe.</t>
         </is>
       </c>
     </row>
@@ -824,7 +832,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>💡 Bitterstoffe (z. B. Angostura) haben eine beruhigende Wirkung auf das Verdauungssystem.</t>
+          <t>Bitterstoffe (z. B. Angostura) haben eine beruhigende Wirkung auf das Verdauungssystem.</t>
         </is>
       </c>
     </row>
@@ -856,7 +864,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>💡 Pfefferminze und Zitrus wirken aktivierend, Lavendel beruhigend. Mehrere Varianten bereithalten.</t>
+          <t>Pfefferminze und Zitrus wirken aktivierend, Lavendel beruhigend. Mehrere Varianten bereithalten.</t>
         </is>
       </c>
     </row>
@@ -888,7 +896,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>💡 Punkt zwischen Daumen und Zeigefinger für 30 – 60 Sekunden fest drücken.</t>
+          <t>Punkt zwischen Daumen und Zeigefinger für 30 – 60 Sekunden fest drücken.</t>
         </is>
       </c>
     </row>
@@ -920,7 +928,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>💡 Kissen als Dämpfer verwenden, wenn kein Aussenbereich vorhanden. Tief einatmen vorher.</t>
+          <t>Kissen als Dämpfer verwenden, wenn kein Aussenbereich vorhanden. Tief einatmen vorher.</t>
         </is>
       </c>
     </row>
@@ -952,7 +960,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>💡 Schon 30 Sekunden kaltes Wasser im Gesicht oder am Handgelenk zeigen Wirkung.</t>
+          <t>Schon 30 Sekunden kaltes Wasser im Gesicht oder am Handgelenk zeigen Wirkung.</t>
         </is>
       </c>
     </row>
@@ -984,7 +992,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>💡 Wenn einschlafen nicht möglich ist, einfach hinlegen und Augen schliessen reicht.</t>
+          <t>Wenn einschlafen nicht möglich ist, einfach hinlegen und Augen schliessen reicht.</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1024,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>💡 Bewusstes Wahrnehmen der Umgebung (Geräusche, Gerüche) verstärkt den Effekt.</t>
+          <t>Bewusstes Wahrnehmen der Umgebung (Geräusche, Gerüche) verstärkt den Effekt.</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1056,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>💡 Laut zusprechen: «Es ist okay. Ich schaffe das. Ich reite das aus.»</t>
+          <t>Laut zusprechen: «Es ist okay. Ich schaffe das. Ich reite das aus.»</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1088,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>💡 Auch Selbstmassage (Hände, Unterarme, Kopfhaut) hat einen messbaren Effekt.</t>
+          <t>Auch Selbstmassage (Hände, Unterarme, Kopfhaut) hat einen messbaren Effekt.</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1120,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>💡 Mit warmem Wasser beginnen, zuletzt auf kalt wechseln und dabei tief ausatmen.</t>
+          <t>Mit warmem Wasser beginnen, zuletzt auf kalt wechseln und dabei tief ausatmen.</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1152,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>💡 Datum, Uhrzeit, Situation, Intensität (0–100 %) und verwendete Skills notieren.</t>
+          <t>Datum, Uhrzeit, Situation, Intensität (0–100 %) und verwendete Skills notieren.</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1184,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>💡 Koffer an einem fixen Ort aufbewahren. Regelmässig nachfüllen.</t>
+          <t>Koffer an einem fixen Ort aufbewahren. Regelmässig nachfüllen.</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1216,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>💡 Aufschreiben: Erst X, dann Y, dann Z. In der Krise kein Nachdenken nötig.</t>
+          <t>Aufschreiben: Erst X, dann Y, dann Z. In der Krise kein Nachdenken nötig.</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1248,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>💡 Gleiche Schlafens- und Aufstehzeit auch am Wochenende einhalten.</t>
+          <t>Gleiche Schlafens- und Aufstehzeit auch am Wochenende einhalten.</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1280,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>💡 Drei Mahlzeiten pro Tag als Minimalziel. Zucker und Koffein reduzieren.</t>
+          <t>Drei Mahlzeiten pro Tag als Minimalziel. Zucker und Koffein reduzieren.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1312,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>💡 Kein Ritual nötig — jede Form des stillen Kontakts mit etwas Grösserem wirkt.</t>
+          <t>Kein Ritual nötig — jede Form des stillen Kontakts mit etwas Grösserem wirkt.</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1344,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>💡 Nicht erzwingen. Auch kleine Dinge zählen: Tageslicht, ein Getränk, eine bequeme Sitzposition.</t>
+          <t>Nicht erzwingen. Auch kleine Dinge zählen: Tageslicht, ein Getränk, eine bequeme Sitzposition.</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1376,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>💡 Wirkt am besten, wenn man bei hoher Anspannung Zeit braucht, bevor man handelt.</t>
+          <t>Wirkt am besten, wenn man bei hoher Anspannung Zeit braucht, bevor man handelt.</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1408,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>💡 Auch Kleinigkeiten: jemandem die Tür aufhalten, eine kurze Nachricht schreiben.</t>
+          <t>Auch Kleinigkeiten: jemandem die Tür aufhalten, eine kurze Nachricht schreiben.</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1440,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>💡 Körperscan oder Atembeobachtung sind gute Einsteigerübungen. Apps wie Insight Timer helfen.</t>
+          <t>Körperscan oder Atembeobachtung sind gute Einsteigerübungen. Apps wie Insight Timer helfen.</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1472,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>💡 Unterarme, Hände und Hals sind besonders empfindlich. Langsam und gezielt streichen.</t>
+          <t>Unterarme, Hände und Hals sind besonders empfindlich. Langsam und gezielt streichen.</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1504,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>💡 Auf verschiedenen Untergründen laufen (Gras, Kies, Holzboden) verstärkt den Effekt.</t>
+          <t>Auf verschiedenen Untergründen laufen (Gras, Kies, Holzboden) verstärkt den Effekt.</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1536,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>💡 Versuchen, im Bild drei Farben, zwei Formen und eine Stimmung zu benennen.</t>
+          <t>Versuchen, im Bild drei Farben, zwei Formen und eine Stimmung zu benennen.</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1568,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>💡 Mit den Fingern auf Brust, Oberschenkel oder Schulter in einem regelmässigen Rhythmus klopfen.</t>
+          <t>Mit den Fingern auf Brust, Oberschenkel oder Schulter in einem regelmässigen Rhythmus klopfen.</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1600,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>💡 Das Ergebnis ist ein Nebenprodukt — der Prozess selbst ist die Therapie.</t>
+          <t>Das Ergebnis ist ein Nebenprodukt — der Prozess selbst ist die Therapie.</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1632,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>💡 Malen nach Zahlen ist besonders geeignet, weil das Ergebnis vorstrukturiert ist — kein Druck.</t>
+          <t>Malen nach Zahlen ist besonders geeignet, weil das Ergebnis vorstrukturiert ist — kein Druck.</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1664,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>💡 Nur eine Schublade oder eine Ecke — kleine Erfolge zählen.</t>
+          <t>Nur eine Schublade oder eine Ecke — kleine Erfolge zählen.</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1696,7 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>💡 Nur umstellen, nicht kaufen. Die Veränderung selbst ist das Ziel.</t>
+          <t>Nur umstellen, nicht kaufen. Die Veränderung selbst ist das Ziel.</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1728,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>💡 Auch das Beobachten (z. B. Fische im Aquarium) hat eine nachweisbar beruhigende Wirkung.</t>
+          <t>Auch das Beobachten (z. B. Fische im Aquarium) hat eine nachweisbar beruhigende Wirkung.</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1760,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>💡 Laut zählen verstärkt den Effekt. Bei Fehler: nochmals von vorne beginnen.</t>
+          <t>Laut zählen verstärkt den Effekt. Bei Fehler: nochmals von vorne beginnen.</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1792,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>💡 Lieblingsshow vorher festlegen, damit in der Krise keine Entscheidung nötig ist.</t>
+          <t>Lieblingsshow vorher festlegen, damit in der Krise keine Entscheidung nötig ist.</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1824,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>💡 Einfach und kostenlos. Bewusstes Wahrnehmen des Gefühls beim Gehen erhöht den Effekt.</t>
+          <t>Einfach und kostenlos. Bewusstes Wahrnehmen des Gefühls beim Gehen erhöht den Effekt.</t>
         </is>
       </c>
     </row>
@@ -1848,7 +1856,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>💡 Vorher festlegen, wen man anruft. Auch eine kurze Nachricht reicht für den ersten Schritt.</t>
+          <t>Vorher festlegen, wen man anruft. Auch eine kurze Nachricht reicht für den ersten Schritt.</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1888,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>💡 So viele Liegestütze wie möglich — bis zur Erschöpfung. Das ist der Punkt.</t>
+          <t>So viele Liegestütze wie möglich — bis zur Erschöpfung. Das ist der Punkt.</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1920,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>💡 Nicht lösen müssen — nur da sein. Das ist genug.</t>
+          <t>Nicht lösen müssen — nur da sein. Das ist genug.</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1952,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>💡 Tief und langsam atmen. Der erste Schreck geht nach 30 Sekunden vorbei.</t>
+          <t>Tief und langsam atmen. Der erste Schreck geht nach 30 Sekunden vorbei.</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1984,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>💡 Nummer im Telefon als «Notfall» speichern. Kontakt vorab über die Rolle informieren.</t>
+          <t>Nummer im Telefon als «Notfall» speichern. Kontakt vorab über die Rolle informieren.</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2016,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>💡 Kein spitzer oder grosser Stein — das Ziel ist Aufmerksamkeit, nicht Schmerz.</t>
+          <t>Kein spitzer oder grosser Stein — das Ziel ist Aufmerksamkeit, nicht Schmerz.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2048,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>💡 Auf Handgelenk, Unterarm oder Hals halten. Bewusst auf die Kälteempfindung konzentrieren.</t>
+          <t>Auf Handgelenk, Unterarm oder Hals halten. Bewusst auf die Kälteempfindung konzentrieren.</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2080,7 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>💡 An Fingerbeere oder Unterarm. Immer als Skill einsetzen, nie als Bestrafung.</t>
+          <t>An Fingerbeere oder Unterarm. Immer als Skill einsetzen, nie als Bestrafung.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2112,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>💡 Nicht zu fest. Das Signal, nicht der Schmerz, ist der Wirkfaktor.</t>
+          <t>Nicht zu fest. Das Signal, nicht der Schmerz, ist der Wirkfaktor.</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2144,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>💡 Keine Antwort erwarten. Nur das Aussprechen ist das Ziel.</t>
+          <t>Keine Antwort erwarten. Nur das Aussprechen ist das Ziel.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2176,7 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>💡 Coolpack: Nacken und Handgelenke. Heisses Bad: 38 – 40 °C, mindestens 15 Minuten.</t>
+          <t>Coolpack: Nacken und Handgelenke. Heisses Bad: 38 – 40 °C, mindestens 15 Minuten.</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2208,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>💡 Oberschenkel, Waden und Rücken. Langsam und mit körperlichem Gewicht arbeiten.</t>
+          <t>Oberschenkel, Waden und Rücken. Langsam und mit körperlichem Gewicht arbeiten.</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2240,7 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>💡 Jumping Jacks, Treppen steigen, Laufen — alles zählt. Ziel: ausser Atem kommen.</t>
+          <t>Jumping Jacks, Treppen steigen, Laufen — alles zählt. Ziel: ausser Atem kommen.</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2272,7 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>💡 Zeitlimit setzen (z. B. 30 Min.) damit Gaming nicht selbst zur Vermeidung wird.</t>
+          <t>Zeitlimit setzen (z. B. 30 Min.) damit Gaming nicht selbst zur Vermeidung wird.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2304,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>💡 Eigenen sicheren Ort im Ruhezustand ausarbeiten (Aussehen, Geräusche, Gefühl), damit er in der Krise abrufbar ist.</t>
+          <t>Eigenen sicheren Ort im Ruhezustand ausarbeiten (Aussehen, Geräusche, Gefühl), damit er in der Krise abrufbar ist.</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2336,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>💡 Die Ausatemphase muss länger sein als die Einatemphase — das ist der Wirkmechanismus.</t>
+          <t>Die Ausatemphase muss länger sein als die Einatemphase — das ist der Wirkmechanismus.</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2368,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>💡 Mit den Händen beginnen: 10 Sek. fest zusammendrücken, dann loslassen und 20 Sek. nachspüren.</t>
+          <t>Mit den Händen beginnen: 10 Sek. fest zusammendrücken, dann loslassen und 20 Sek. nachspüren.</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2400,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>💡 Ein eigenes «Freude-Album» auf dem Handy anlegen, das jederzeit verfügbar ist.</t>
+          <t>Ein eigenes «Freude-Album» auf dem Handy anlegen, das jederzeit verfügbar ist.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2432,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>💡 Thema wählen (z. B. Urlaub, Freunde, Natur) und 15 – 20 Fotos auswählen.</t>
+          <t>Thema wählen (z. B. Urlaub, Freunde, Natur) und 15 – 20 Fotos auswählen.</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2464,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>💡 So genau wie möglich: nicht «schlecht», sondern «ich fühle Angst und Hilflosigkeit».</t>
+          <t>So genau wie möglich: nicht «schlecht», sondern «ich fühle Angst und Hilflosigkeit».</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2496,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>💡 Keine Gedanken wegdrängen — sie beobachten wie Wolken, die vorbeizeigen.</t>
+          <t>Keine Gedanken wegdrängen — sie beobachten wie Wolken, die vorbeizeigen.</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2528,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>💡 Auch 10 Minuten sanftes Yoga (z. B. Kind-Pose, Vorwärtsbeuge) haben einen messbaren Effekt.</t>
+          <t>Auch 10 Minuten sanftes Yoga (z. B. Kind-Pose, Vorwärtsbeuge) haben einen messbaren Effekt.</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2560,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>💡 Satz: «Es ist, wie es ist. Ich kann die Vergangenheit nicht ändern. Was kann ich jetzt tun?»</t>
+          <t>Satz: «Es ist, wie es ist. Ich kann die Vergangenheit nicht ändern. Was kann ich jetzt tun?»</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2592,7 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>💡 Nicht für immer — nur für die nächste Stunde. Dann neu entscheiden.</t>
+          <t>Nicht für immer — nur für die nächste Stunde. Dann neu entscheiden.</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2624,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>💡 Kein Perfektionismus. Stichworte genügen. Das Schreiben selbst ist der Wirkfaktor.</t>
+          <t>Kein Perfektionismus. Stichworte genügen. Das Schreiben selbst ist der Wirkfaktor.</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2656,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>💡 Skala 0 – 10 nutzen für Stimmung, Anspannung und Energie — dreimal täglich.</t>
+          <t>Skala 0 – 10 nutzen für Stimmung, Anspannung und Energie — dreimal täglich.</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2688,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>💡 Erst 3 Dinge sehen benennen, dann 3 hören, dann 3 am Körper spüren.</t>
+          <t>Erst 3 Dinge sehen benennen, dann 3 hören, dann 3 am Körper spüren.</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2720,7 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>💡 Maximal 3 – 5 Aufgaben. Sehr kleine Schritte — z. B. «ein Glas Wasser trinken» zählt.</t>
+          <t>Maximal 3 – 5 Aufgaben. Sehr kleine Schritte — z. B. «ein Glas Wasser trinken» zählt.</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2752,7 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>💡 Alte Favoriten wirken besser als Neues — die Vertrautheit ist der beruhigende Faktor.</t>
+          <t>Alte Favoriten wirken besser als Neues — die Vertrautheit ist der beruhigende Faktor.</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2784,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>💡 Eine Playlist für ruhige Momente vorab zusammenstellen.</t>
+          <t>Eine Playlist für ruhige Momente vorab zusammenstellen.</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2816,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>💡 Der Schwierigkeitsgrad sollte herausfordernd, aber lösbar sein — Frust wäre kontraproduktiv.</t>
+          <t>Der Schwierigkeitsgrad sollte herausfordernd, aber lösbar sein — Frust wäre kontraproduktiv.</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2848,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>💡 Den Cube im Ruhezustand lösen lernen — dann ist er in stressigen Momenten abrufbar.</t>
+          <t>Den Cube im Ruhezustand lösen lernen — dann ist er in stressigen Momenten abrufbar.</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2880,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>💡 Rückwärts buchstabieren erhöht den kognitiven Aufwand deutlich.</t>
+          <t>Rückwärts buchstabieren erhöht den kognitiven Aufwand deutlich.</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2912,7 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>💡 Auch das Zeichnen von einfachen Formen mit der anderen Hand reicht aus.</t>
+          <t>Auch das Zeichnen von einfachen Formen mit der anderen Hand reicht aus.</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2944,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>💡 Leichtes, vertrautes Material wählen. Kein Selbsthilfebuch in der Krise.</t>
+          <t>Leichtes, vertrautes Material wählen. Kein Selbsthilfebuch in der Krise.</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2976,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>💡 Kurze Gedichte oder Liedstrophen beginnen. Wiederholung ist der Schlüssel.</t>
+          <t>Kurze Gedichte oder Liedstrophen beginnen. Wiederholung ist der Schlüssel.</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3008,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>💡 Augen schliessen während des Balancierens erhöht die Anforderung deutlich.</t>
+          <t>Augen schliessen während des Balancierens erhöht die Anforderung deutlich.</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3040,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>💡 Kleine, machbare Aufgaben wählen — der Nagel im Regal, der Knopf am Hemd.</t>
+          <t>Kleine, machbare Aufgaben wählen — der Nagel im Regal, der Knopf am Hemd.</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3072,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>💡 Lieblingsgericht kochen. Der Prozess ist die Therapie, das Essen der Bonus.</t>
+          <t>Lieblingsgericht kochen. Der Prozess ist die Therapie, das Essen der Bonus.</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3104,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>💡 Handy weglegen. Jeden Bissen 10 – 15 Mal kauen und bewusst wahrnehmen.</t>
+          <t>Handy weglegen. Jeden Bissen 10 – 15 Mal kauen und bewusst wahrnehmen.</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3136,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>💡 Schwierigkeitsgrad anpassen: In der Erholung lieber einfacher beginnen.</t>
+          <t>Schwierigkeitsgrad anpassen: In der Erholung lieber einfacher beginnen.</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3168,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>💡 Schwierigkeitsgrad wählen, der Herausforderung bietet, aber nicht frustriert.</t>
+          <t>Schwierigkeitsgrad wählen, der Herausforderung bietet, aber nicht frustriert.</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3200,7 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>💡 Zeitung oder App. Das Erstellen eigener Rätsel für andere ist ein höheres Ziel.</t>
+          <t>Zeitung oder App. Das Erstellen eigener Rätsel für andere ist ein höheres Ziel.</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3232,7 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>💡 Thema wählen: z. B. «Alles in Blau» oder «Dinge auf dem Boden». Handykamera reicht.</t>
+          <t>Thema wählen: z. B. «Alles in Blau» oder «Dinge auf dem Boden». Handykamera reicht.</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3264,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>💡 Formen in Wolken suchen oder einfach dem Ziehen folgen ohne zu bewerten.</t>
+          <t>Formen in Wolken suchen oder einfach dem Ziehen folgen ohne zu bewerten.</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3296,7 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>💡 Nach dem Regen nach draussengehen. Frische Erde riechen (Petrichor) wirkt besonders.</t>
+          <t>Nach dem Regen nach draussengehen. Frische Erde riechen (Petrichor) wirkt besonders.</t>
         </is>
       </c>
     </row>
@@ -3320,7 +3328,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>💡 Eine Hand auf den Bauch legen und nur das Heben und Senken wahrnehmen.</t>
+          <t>Eine Hand auf den Bauch legen und nur das Heben und Senken wahrnehmen.</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3360,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>💡 Metronom-App auf 60 BPM einstellen. Die Synchronisierung der eigenen Atmung verstärkt den Effekt.</t>
+          <t>Metronom-App auf 60 BPM einstellen. Die Synchronisierung der eigenen Atmung verstärkt den Effekt.</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3392,7 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>💡 Einfach sitzen und schauen, ohne etwas tun zu müssen. Das ist genug.</t>
+          <t>Einfach sitzen und schauen, ohne etwas tun zu müssen. Das ist genug.</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3424,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>💡 Den Finger langsam von links nach rechts bewegen und mit den Augen folgen, 20 – 30 Sekunden.</t>
+          <t>Den Finger langsam von links nach rechts bewegen und mit den Augen folgen, 20 – 30 Sekunden.</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3456,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>💡 Ohrsstöpsel oder Kopfhörer verwenden. YouTube oder Entspannungs-Apps haben stundenlange Aufnahmen.</t>
+          <t>Ohrsstöpsel oder Kopfhörer verwenden. YouTube oder Entspannungs-Apps haben stundenlange Aufnahmen.</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3488,7 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>💡 Lächeln in den Spiegel schauen, 30 Sekunden halten. Wirkt besser als man denkt.</t>
+          <t>Lächeln in den Spiegel schauen, 30 Sekunden halten. Wirkt besser als man denkt.</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3520,7 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>💡 Mindestens 10 Minuten. Der Effekt baut sich mit der Zeit auf.</t>
+          <t>Mindestens 10 Minuten. Der Effekt baut sich mit der Zeit auf.</t>
         </is>
       </c>
     </row>
@@ -3544,7 +3552,7 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>💡 Kerze, Kamin oder Lagerfeuer. Auch ein Feuer-Video auf dem Bildschirm hat eine messbare Wirkung.</t>
+          <t>Kerze, Kamin oder Lagerfeuer. Auch ein Feuer-Video auf dem Bildschirm hat eine messbare Wirkung.</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3584,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>💡 Handy in der Tasche lassen. Bei jedem Schritt bewusst den Bodenkontakt wahrnehmen.</t>
+          <t>Handy in der Tasche lassen. Bei jedem Schritt bewusst den Bodenkontakt wahrnehmen.</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3616,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>💡 Basilikum, Thymian, Minze, Rosmarin — blind oder mit geschlossenen Augen erraten.</t>
+          <t>Basilikum, Thymian, Minze, Rosmarin — blind oder mit geschlossenen Augen erraten.</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3648,7 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>💡 Frische Zitrone, Lavendel oder Rosen eignen sich besonders gut. Tief einatmen, 5 – 10 Atemzüge.</t>
+          <t>Frische Zitrone, Lavendel oder Rosen eignen sich besonders gut. Tief einatmen, 5 – 10 Atemzüge.</t>
         </is>
       </c>
     </row>
@@ -3672,11 +3680,12 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>💡 «Power Pose»: 2 Minuten mit breitem Stand und auf Hüfte gestützten Händen stehen.</t>
+          <t>«Power Pose»: 2 Minuten mit breitem Stand und auf Hüfte gestützten Händen stehen.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F101"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Stufe" error="Bitte Hoch, Mittel oder Tief wählen." promptTitle="Stufe" prompt="Hoch / Mittel / Tief" type="list">
       <formula1>"Hoch,Mittel,Tief"</formula1>
@@ -3874,6 +3883,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H4"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Stufe" error="Bitte Hoch, Mittel oder Tief wählen." promptTitle="Stufe" prompt="Hoch / Mittel / Tief" type="list">
       <formula1>"Hoch,Mittel,Tief"</formula1>
@@ -4068,6 +4078,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C10"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Stufe" error="Bitte Hoch, Mittel oder Tief wählen." promptTitle="Stufe" prompt="Hoch / Mittel / Tief" type="list">
       <formula1>"Hoch,Mittel,Tief"</formula1>

</xml_diff>